<commit_message>
- Made sure #8 was fixed. - updated list_widgets_fields.xlsx
</commit_message>
<xml_diff>
--- a/gui/resources/list_widgets_fields.xlsx
+++ b/gui/resources/list_widgets_fields.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24809"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26505"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MKhos\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\vcams\gui\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF383C4B-E340-449A-8E4E-F83B56893EEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885512A9-1679-48EE-B0E2-8C4BD2A8ED70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8B64B68D-724C-4491-A6CC-F87AC3DD731E}"/>
   </bookViews>
@@ -20,20 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="80">
   <si>
     <t>Section</t>
   </si>
@@ -255,6 +247,24 @@
   </si>
   <si>
     <t>tpms_fill_value</t>
+  </si>
+  <si>
+    <t>run_export_button</t>
+  </si>
+  <si>
+    <t>run_create_model_button</t>
+  </si>
+  <si>
+    <t>Run</t>
+  </si>
+  <si>
+    <t>run_open_dir_button</t>
+  </si>
+  <si>
+    <t>QPushButton</t>
+  </si>
+  <si>
+    <t>log_field</t>
   </si>
 </sst>
 </file>
@@ -307,6 +317,24 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}" name="Table1" displayName="Table1" ref="A1:D36" totalsRowShown="0">
+  <autoFilter ref="A1:D36" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{67129673-70B6-4E64-96E4-F0D46A127B44}" name="Section"/>
+    <tableColumn id="2" xr3:uid="{102936D2-304C-449A-9085-A82C8887ABFE}" name="Key in Config File"/>
+    <tableColumn id="3" xr3:uid="{AAD74926-C818-4DA9-8732-30E630982058}" name="Object Name"/>
+    <tableColumn id="4" xr3:uid="{ED1AF045-1B1D-4EE1-BAA2-EBD21777CF56}" name="Object Class"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1007,64 +1035,123 @@
         <v>68</v>
       </c>
     </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" t="s">
+        <v>55</v>
+      </c>
+      <c r="C31" t="s">
+        <v>54</v>
+      </c>
+      <c r="D31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" t="s">
+        <v>26</v>
+      </c>
+    </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="B33" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="C33" t="s">
-        <v>49</v>
+        <v>74</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="B34" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="D34" t="s">
-        <v>26</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="C35" t="s">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="D35" t="s">
-        <v>36</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="B36" t="s">
-        <v>57</v>
+        <v>79</v>
       </c>
       <c r="C36" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="D36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
- added single and multi image to main_window.ui.
</commit_message>
<xml_diff>
--- a/gui/resources/list_widgets_fields.xlsx
+++ b/gui/resources/list_widgets_fields.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26505"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26602"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\vcams\gui\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885512A9-1679-48EE-B0E2-8C4BD2A8ED70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA70BEE4-ADCF-4C4B-A2F2-B6EF57C9BD06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8B64B68D-724C-4491-A6CC-F87AC3DD731E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="92">
   <si>
     <t>Section</t>
   </si>
@@ -265,14 +265,58 @@
   </si>
   <si>
     <t>log_field</t>
+  </si>
+  <si>
+    <t>single_image_path_field</t>
+  </si>
+  <si>
+    <t>single_image_path</t>
+  </si>
+  <si>
+    <t>single_image_scale_field</t>
+  </si>
+  <si>
+    <t>single_image_scale</t>
+  </si>
+  <si>
+    <t>single_image_denoise_checkbox</t>
+  </si>
+  <si>
+    <t>single_image_denoise</t>
+  </si>
+  <si>
+    <t>multi_image_path</t>
+  </si>
+  <si>
+    <t>multi_image_path_field</t>
+  </si>
+  <si>
+    <t>multi_image_scale_field</t>
+  </si>
+  <si>
+    <t>multi_image_denoise_checkbox</t>
+  </si>
+  <si>
+    <t>multi_image_scale</t>
+  </si>
+  <si>
+    <t>multi_image_denoise</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -300,8 +344,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -320,8 +365,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}" name="Table1" displayName="Table1" ref="A1:D36" totalsRowShown="0">
-  <autoFilter ref="A1:D36" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}" name="Table1" displayName="Table1" ref="A1:D42" totalsRowShown="0">
+  <autoFilter ref="A1:D42" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -634,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D6988C3-CC26-4EA8-8CC8-914DEE59DEFC}">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.5546875" customWidth="1"/>
@@ -1011,53 +1056,53 @@
       <c r="A27" t="s">
         <v>58</v>
       </c>
-      <c r="B27" t="s">
-        <v>67</v>
+      <c r="B27" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="D27" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>58</v>
       </c>
-      <c r="B28" t="s">
-        <v>69</v>
+      <c r="B28" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="D28" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>50</v>
-      </c>
-      <c r="B29" t="s">
-        <v>51</v>
+        <v>58</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>84</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>50</v>
-      </c>
-      <c r="B30" t="s">
-        <v>53</v>
+        <v>58</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="C30" t="s">
-        <v>52</v>
+        <v>87</v>
       </c>
       <c r="D30" t="s">
         <v>26</v>
@@ -1065,85 +1110,169 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>50</v>
-      </c>
-      <c r="B31" t="s">
-        <v>55</v>
+        <v>58</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="C31" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="D31" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" t="s">
-        <v>57</v>
+        <v>58</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="C32" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="D32" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="B33" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C33" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="D33" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="B35" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="C35" t="s">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="D35" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" t="s">
+        <v>52</v>
+      </c>
+      <c r="D36" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C37" t="s">
+        <v>54</v>
+      </c>
+      <c r="D37" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" t="s">
+        <v>56</v>
+      </c>
+      <c r="D38" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
         <v>76</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B39" t="s">
+        <v>74</v>
+      </c>
+      <c r="C39" t="s">
+        <v>74</v>
+      </c>
+      <c r="D39" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" t="s">
+        <v>75</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>76</v>
+      </c>
+      <c r="B41" t="s">
+        <v>77</v>
+      </c>
+      <c r="C41" t="s">
+        <v>77</v>
+      </c>
+      <c r="D41" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" t="s">
         <v>79</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C42" t="s">
         <v>79</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D42" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added a working version of the random modeling mode to the GUI.
</commit_message>
<xml_diff>
--- a/gui/resources/list_widgets_fields.xlsx
+++ b/gui/resources/list_widgets_fields.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26610"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28011"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\vcams\gui\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31B0D18-5D79-433E-B506-54FDB5DA8631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9FB3120-9B0E-44BD-8C10-CF71988CCB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8B64B68D-724C-4491-A6CC-F87AC3DD731E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="96">
   <si>
     <t>Section</t>
   </si>
@@ -301,6 +301,18 @@
   </si>
   <si>
     <t>multi_image_denoise</t>
+  </si>
+  <si>
+    <t>random_phase_matcode</t>
+  </si>
+  <si>
+    <t>random_phase_fraction</t>
+  </si>
+  <si>
+    <t>random_phase_fraction_field</t>
+  </si>
+  <si>
+    <t>random_phase_matcode_field</t>
   </si>
 </sst>
 </file>
@@ -336,9 +348,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -357,8 +368,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}" name="Table1" displayName="Table1" ref="A1:D42" totalsRowShown="0">
-  <autoFilter ref="A1:D42" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}" name="Table1" displayName="Table1" ref="A1:D44" totalsRowShown="0">
+  <autoFilter ref="A1:D44" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -671,12 +682,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D6988C3-CC26-4EA8-8CC8-914DEE59DEFC}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.5546875" customWidth="1"/>
-    <col min="2" max="2" width="24.88671875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" customWidth="1"/>
+    <col min="3" max="3" width="35.21875" customWidth="1"/>
     <col min="4" max="4" width="34.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -993,13 +1004,13 @@
         <v>58</v>
       </c>
       <c r="B23" t="s">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="D23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1007,10 +1018,10 @@
         <v>58</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="D24" t="s">
         <v>26</v>
@@ -1021,13 +1032,13 @@
         <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1035,10 +1046,10 @@
         <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C26" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D26" t="s">
         <v>26</v>
@@ -1048,11 +1059,11 @@
       <c r="A27" t="s">
         <v>58</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>81</v>
+      <c r="B27" t="s">
+        <v>65</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="D27" t="s">
         <v>26</v>
@@ -1062,11 +1073,11 @@
       <c r="A28" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>83</v>
+      <c r="B28" t="s">
+        <v>73</v>
       </c>
       <c r="C28" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D28" t="s">
         <v>26</v>
@@ -1076,25 +1087,25 @@
       <c r="A29" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>85</v>
+      <c r="B29" t="s">
+        <v>81</v>
       </c>
       <c r="C29" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D29" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>86</v>
+      <c r="B30" t="s">
+        <v>83</v>
       </c>
       <c r="C30" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D30" t="s">
         <v>26</v>
@@ -1104,42 +1115,42 @@
       <c r="A31" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>90</v>
+      <c r="B31" t="s">
+        <v>85</v>
       </c>
       <c r="C31" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D31" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>58</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>91</v>
+      <c r="B32" t="s">
+        <v>86</v>
       </c>
       <c r="C32" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D32" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>67</v>
+      <c r="B33" t="s">
+        <v>90</v>
       </c>
       <c r="C33" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="D33" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -1147,41 +1158,41 @@
         <v>58</v>
       </c>
       <c r="B34" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="D34" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B35" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="C35" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="D35" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B36" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="C36" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="D36" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
@@ -1189,13 +1200,13 @@
         <v>50</v>
       </c>
       <c r="B37" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C37" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D37" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
@@ -1203,10 +1214,10 @@
         <v>50</v>
       </c>
       <c r="B38" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C38" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D38" t="s">
         <v>26</v>
@@ -1214,30 +1225,30 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="B39" t="s">
-        <v>74</v>
+        <v>55</v>
       </c>
       <c r="C39" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="D39" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="C40" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="D40" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
@@ -1245,10 +1256,10 @@
         <v>76</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C41" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D41" t="s">
         <v>78</v>
@@ -1259,12 +1270,40 @@
         <v>76</v>
       </c>
       <c r="B42" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>76</v>
+      </c>
+      <c r="B43" t="s">
+        <v>77</v>
+      </c>
+      <c r="C43" t="s">
+        <v>77</v>
+      </c>
+      <c r="D43" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>76</v>
+      </c>
+      <c r="B44" t="s">
         <v>79</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C44" t="s">
         <v>79</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D44" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
created the fields to the ui and added import/export logic.
</commit_message>
<xml_diff>
--- a/gui/resources/list_widgets_fields.xlsx
+++ b/gui/resources/list_widgets_fields.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29011"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\vcams\gui\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9FB3120-9B0E-44BD-8C10-CF71988CCB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0C4E96-175B-4F99-B29E-DD77B0F86F89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8B64B68D-724C-4491-A6CC-F87AC3DD731E}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="104">
   <si>
     <t>Section</t>
   </si>
@@ -313,6 +313,30 @@
   </si>
   <si>
     <t>random_phase_matcode_field</t>
+  </si>
+  <si>
+    <t>single_image_thresh_mode</t>
+  </si>
+  <si>
+    <t>single_image_thresh_value</t>
+  </si>
+  <si>
+    <t>single_image_thresh_value_field</t>
+  </si>
+  <si>
+    <t>multi_image_thresh_mode</t>
+  </si>
+  <si>
+    <t>multi_image_thresh_value</t>
+  </si>
+  <si>
+    <t>multi_image_thresh_value_field</t>
+  </si>
+  <si>
+    <t>single_image_thresh_mode_combo</t>
+  </si>
+  <si>
+    <t>multi_image_thresh_mode_combo</t>
   </si>
 </sst>
 </file>
@@ -368,8 +392,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}" name="Table1" displayName="Table1" ref="A1:D44" totalsRowShown="0">
-  <autoFilter ref="A1:D44" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}" name="Table1" displayName="Table1" ref="A1:D48" totalsRowShown="0">
+  <autoFilter ref="A1:D48" xr:uid="{790EF0F8-926A-4EC3-B95E-939E58EADA65}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -682,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D6988C3-CC26-4EA8-8CC8-914DEE59DEFC}">
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.5546875" customWidth="1"/>
@@ -1116,13 +1140,13 @@
         <v>58</v>
       </c>
       <c r="B31" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="C31" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="D31" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -1130,10 +1154,10 @@
         <v>58</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="C32" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="D32" t="s">
         <v>26</v>
@@ -1144,13 +1168,13 @@
         <v>58</v>
       </c>
       <c r="B33" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D33" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -1158,13 +1182,13 @@
         <v>58</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D34" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -1172,13 +1196,13 @@
         <v>58</v>
       </c>
       <c r="B35" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C35" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="D35" t="s">
-        <v>68</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -1186,24 +1210,24 @@
         <v>58</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>100</v>
       </c>
       <c r="C37" t="s">
-        <v>49</v>
+        <v>101</v>
       </c>
       <c r="D37" t="s">
         <v>26</v>
@@ -1211,99 +1235,155 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B38" t="s">
-        <v>53</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="D38" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B39" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="D39" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B40" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="D40" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>74</v>
+        <v>51</v>
       </c>
       <c r="C41" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="D41" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="B42" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C42" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
       <c r="D42" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="B43" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="C43" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="D43" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" t="s">
+        <v>56</v>
+      </c>
+      <c r="D44" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
         <v>76</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
+        <v>74</v>
+      </c>
+      <c r="C45" t="s">
+        <v>74</v>
+      </c>
+      <c r="D45" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>76</v>
+      </c>
+      <c r="B46" t="s">
+        <v>75</v>
+      </c>
+      <c r="C46" t="s">
+        <v>75</v>
+      </c>
+      <c r="D46" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>76</v>
+      </c>
+      <c r="B47" t="s">
+        <v>77</v>
+      </c>
+      <c r="C47" t="s">
+        <v>77</v>
+      </c>
+      <c r="D47" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>76</v>
+      </c>
+      <c r="B48" t="s">
         <v>79</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C48" t="s">
         <v>79</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D48" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>